<commit_message>
update vendor B compiler spec
</commit_message>
<xml_diff>
--- a/Template/KWS8_SOW.xlsx
+++ b/Template/KWS8_SOW.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\msys64\home\Administrator\github\MD_Group\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A6AF64F-2283-418D-83D0-D6FAF843B79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C9AA96-1CAD-47F9-B970-0F26B7E8B12A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3615" yWindow="2385" windowWidth="30915" windowHeight="17520" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3615" yWindow="2385" windowWidth="30915" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 2" sheetId="4" r:id="rId1"/>
     <sheet name="Table 3 (1)" sheetId="18" r:id="rId2"/>
-    <sheet name="Table 3" sheetId="3" r:id="rId3"/>
-    <sheet name="Table4 (1)" sheetId="2" r:id="rId4"/>
-    <sheet name="Table4 (2)" sheetId="5" r:id="rId5"/>
-    <sheet name="Table4 (3)" sheetId="6" r:id="rId6"/>
-    <sheet name="Table4 (4)" sheetId="7" r:id="rId7"/>
-    <sheet name="Table4 (5)" sheetId="8" r:id="rId8"/>
-    <sheet name="Table4 (6)" sheetId="9" r:id="rId9"/>
-    <sheet name="Table4 (7)" sheetId="10" r:id="rId10"/>
-    <sheet name="Table4 (8)" sheetId="11" r:id="rId11"/>
-    <sheet name="Table4 (9)" sheetId="12" r:id="rId12"/>
-    <sheet name="Table 5" sheetId="13" r:id="rId13"/>
-    <sheet name="Table 6" sheetId="14" r:id="rId14"/>
-    <sheet name="Table 7" sheetId="15" r:id="rId15"/>
-    <sheet name="Table 8" sheetId="16" r:id="rId16"/>
-    <sheet name="Table 9" sheetId="17" r:id="rId17"/>
+    <sheet name="Table 3 (2)" sheetId="19" r:id="rId3"/>
+    <sheet name="Table 3" sheetId="3" r:id="rId4"/>
+    <sheet name="Table4 (1)" sheetId="2" r:id="rId5"/>
+    <sheet name="Table4 (2)" sheetId="5" r:id="rId6"/>
+    <sheet name="Table4 (3)" sheetId="6" r:id="rId7"/>
+    <sheet name="Table4 (4)" sheetId="7" r:id="rId8"/>
+    <sheet name="Table4 (5)" sheetId="8" r:id="rId9"/>
+    <sheet name="Table4 (6)" sheetId="9" r:id="rId10"/>
+    <sheet name="Table4 (7)" sheetId="10" r:id="rId11"/>
+    <sheet name="Table4 (8)" sheetId="11" r:id="rId12"/>
+    <sheet name="Table4 (9)" sheetId="12" r:id="rId13"/>
+    <sheet name="Table 5" sheetId="13" r:id="rId14"/>
+    <sheet name="Table 6" sheetId="14" r:id="rId15"/>
+    <sheet name="Table 7" sheetId="15" r:id="rId16"/>
+    <sheet name="Table 8" sheetId="16" r:id="rId17"/>
+    <sheet name="Table 9" sheetId="17" r:id="rId18"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="263">
   <si>
     <t>Table Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -863,6 +864,86 @@
   </si>
   <si>
     <t>0.1080</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Table: Vendor B Memory Compiler 定义</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>One Port Register File</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Two Port Register File</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dual Port SRAM Compiler</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ROM Compiler</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ultra High Density Two Port SRAM Compiler</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Single Port SRAM Compiler</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Density Single Port Single Bank SRAM Compiler with Smaller HD cell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Density Single Port Multi Bank SRAM Compiler with Smaller HD cell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Performace Single Port Single Bank SRAM Compiler with Smaller HC cell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Performace Single Port Multi Bank SRAM Compiler with Smaller HC cell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Performace L1 Cache with HC cell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P13</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>P14</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D1300 8T2P_2FIN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D0734 HD6T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Density Single Port Single Bank SRAM Compiler with HD cell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High Density Single Port Multi Bank SRAM Compiler with HD cell</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1113,6 +1194,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1120,12 +1207,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1492,6 +1573,418 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A658CE8-E02B-4E77-964D-75024B4BFBF4}">
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="53.375" customWidth="1"/>
+    <col min="5" max="5" width="11.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2">
+        <v>32</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1024</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2">
+        <v>320</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="17"/>
+      <c r="B3" s="2">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2">
+        <v>64</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2048</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>8</v>
+      </c>
+      <c r="I3" s="2">
+        <v>320</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="17"/>
+      <c r="B4" s="2">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2">
+        <v>128</v>
+      </c>
+      <c r="F4" s="2">
+        <v>4096</v>
+      </c>
+      <c r="G4" s="2">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2">
+        <v>8</v>
+      </c>
+      <c r="I4" s="2">
+        <v>320</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="17"/>
+      <c r="B5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2">
+        <v>256</v>
+      </c>
+      <c r="F5" s="2">
+        <v>4096</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>8</v>
+      </c>
+      <c r="I5" s="2">
+        <v>320</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="17"/>
+      <c r="B6" s="2">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2">
+        <v>64</v>
+      </c>
+      <c r="F6" s="2">
+        <v>2048</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2">
+        <v>8</v>
+      </c>
+      <c r="I6" s="2">
+        <v>160</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="17"/>
+      <c r="B7" s="2">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2">
+        <v>32</v>
+      </c>
+      <c r="E7" s="2">
+        <v>128</v>
+      </c>
+      <c r="F7" s="2">
+        <v>4096</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2">
+        <v>8</v>
+      </c>
+      <c r="I7" s="2">
+        <v>160</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="17"/>
+      <c r="B8" s="2">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2">
+        <v>32</v>
+      </c>
+      <c r="E8" s="2">
+        <v>256</v>
+      </c>
+      <c r="F8" s="2">
+        <v>8192</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2">
+        <v>8</v>
+      </c>
+      <c r="I8" s="2">
+        <v>160</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" s="17"/>
+      <c r="B9" s="2">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2">
+        <v>32</v>
+      </c>
+      <c r="E9" s="2">
+        <v>512</v>
+      </c>
+      <c r="F9" s="2">
+        <v>8192</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2">
+        <v>8</v>
+      </c>
+      <c r="I9" s="2">
+        <v>160</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="17"/>
+      <c r="B10" s="2">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>64</v>
+      </c>
+      <c r="E10" s="2">
+        <v>128</v>
+      </c>
+      <c r="F10" s="2">
+        <v>4096</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2">
+        <v>8</v>
+      </c>
+      <c r="I10" s="2">
+        <v>80</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="17"/>
+      <c r="B11" s="2">
+        <v>16</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2">
+        <v>64</v>
+      </c>
+      <c r="E11" s="2">
+        <v>256</v>
+      </c>
+      <c r="F11" s="2">
+        <v>8192</v>
+      </c>
+      <c r="G11" s="2">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2">
+        <v>8</v>
+      </c>
+      <c r="I11" s="2">
+        <v>80</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="17"/>
+      <c r="B12" s="2">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2">
+        <v>4</v>
+      </c>
+      <c r="D12" s="2">
+        <v>64</v>
+      </c>
+      <c r="E12" s="2">
+        <v>512</v>
+      </c>
+      <c r="F12" s="2">
+        <v>16384</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2">
+        <v>8</v>
+      </c>
+      <c r="I12" s="2">
+        <v>80</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" s="17"/>
+      <c r="B13" s="2">
+        <v>16</v>
+      </c>
+      <c r="C13" s="2">
+        <v>8</v>
+      </c>
+      <c r="D13" s="2">
+        <v>64</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1024</v>
+      </c>
+      <c r="F13" s="2">
+        <v>16384</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>8</v>
+      </c>
+      <c r="I13" s="2">
+        <v>80</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A13"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9493FFE-5CE4-4A39-8210-DFC5C0C18AD9}">
   <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -1533,7 +2026,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="16" t="s">
         <v>48</v>
       </c>
       <c r="B2" s="2">
@@ -1565,7 +2058,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="20"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="2">
         <v>8</v>
       </c>
@@ -1595,7 +2088,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="20"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="2">
         <v>8</v>
       </c>
@@ -1625,7 +2118,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="20"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="2">
         <v>8</v>
       </c>
@@ -1655,7 +2148,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="2">
         <v>16</v>
       </c>
@@ -1685,7 +2178,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="2">
         <v>16</v>
       </c>
@@ -1715,7 +2208,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
+      <c r="A8" s="17"/>
       <c r="B8" s="2">
         <v>16</v>
       </c>
@@ -1745,7 +2238,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
+      <c r="A9" s="17"/>
       <c r="B9" s="2">
         <v>16</v>
       </c>
@@ -1775,7 +2268,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="20"/>
+      <c r="A10" s="17"/>
       <c r="B10" s="2">
         <v>32</v>
       </c>
@@ -1805,7 +2298,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
+      <c r="A11" s="17"/>
       <c r="B11" s="2">
         <v>32</v>
       </c>
@@ -1835,7 +2328,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="20"/>
+      <c r="A12" s="17"/>
       <c r="B12" s="2">
         <v>32</v>
       </c>
@@ -1865,7 +2358,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="20"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="2">
         <v>32</v>
       </c>
@@ -1895,7 +2388,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="20"/>
+      <c r="A14" s="17"/>
       <c r="B14" s="2">
         <v>64</v>
       </c>
@@ -1925,7 +2418,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="20"/>
+      <c r="A15" s="17"/>
       <c r="B15" s="2">
         <v>64</v>
       </c>
@@ -1955,7 +2448,7 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="20"/>
+      <c r="A16" s="17"/>
       <c r="B16" s="2">
         <v>64</v>
       </c>
@@ -1985,7 +2478,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="20"/>
+      <c r="A17" s="17"/>
       <c r="B17" s="2">
         <v>64</v>
       </c>
@@ -2023,7 +2516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CB24599-813B-4A17-9A91-43B0216E65F3}">
   <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -2065,7 +2558,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="16" t="s">
         <v>49</v>
       </c>
       <c r="B2" s="2">
@@ -2097,7 +2590,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="20"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="2">
         <v>4</v>
       </c>
@@ -2127,7 +2620,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="20"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="2">
         <v>4</v>
       </c>
@@ -2157,7 +2650,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="20"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="2">
         <v>4</v>
       </c>
@@ -2187,7 +2680,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="2">
         <v>8</v>
       </c>
@@ -2217,7 +2710,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="2">
         <v>8</v>
       </c>
@@ -2247,7 +2740,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
+      <c r="A8" s="17"/>
       <c r="B8" s="2">
         <v>8</v>
       </c>
@@ -2277,7 +2770,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
+      <c r="A9" s="17"/>
       <c r="B9" s="2">
         <v>8</v>
       </c>
@@ -2307,7 +2800,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="20"/>
+      <c r="A10" s="17"/>
       <c r="B10" s="2">
         <v>16</v>
       </c>
@@ -2337,7 +2830,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
+      <c r="A11" s="17"/>
       <c r="B11" s="2">
         <v>16</v>
       </c>
@@ -2367,7 +2860,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="20"/>
+      <c r="A12" s="17"/>
       <c r="B12" s="2">
         <v>16</v>
       </c>
@@ -2397,7 +2890,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="20"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="2">
         <v>16</v>
       </c>
@@ -2435,7 +2928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6CF4CE9-FED6-4574-A0AD-D97C88CA816A}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -2477,7 +2970,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B2" s="2">
@@ -2509,7 +3002,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="2">
         <v>4</v>
       </c>
@@ -2547,7 +3040,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F23BCBF9-16F4-4CFD-946E-F8D5918F6152}">
   <dimension ref="A1:G56"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -2581,7 +3074,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>169</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -2604,7 +3097,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="11" t="s">
         <v>72</v>
       </c>
@@ -2625,7 +3118,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="11" t="s">
         <v>73</v>
       </c>
@@ -2646,7 +3139,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="11" t="s">
         <v>75</v>
       </c>
@@ -2667,7 +3160,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="16"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="11" t="s">
         <v>77</v>
       </c>
@@ -2688,7 +3181,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="11" t="s">
         <v>78</v>
       </c>
@@ -2709,7 +3202,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="11" t="s">
         <v>79</v>
       </c>
@@ -2730,7 +3223,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="11" t="s">
         <v>82</v>
       </c>
@@ -2751,7 +3244,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="16"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="11" t="s">
         <v>83</v>
       </c>
@@ -2772,7 +3265,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="16"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="11" t="s">
         <v>84</v>
       </c>
@@ -2793,7 +3286,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="16"/>
+      <c r="A12" s="18"/>
       <c r="B12" s="11" t="s">
         <v>85</v>
       </c>
@@ -2814,7 +3307,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="16"/>
+      <c r="A13" s="18"/>
       <c r="B13" s="11" t="s">
         <v>86</v>
       </c>
@@ -2835,7 +3328,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="16"/>
+      <c r="A14" s="18"/>
       <c r="B14" s="11" t="s">
         <v>87</v>
       </c>
@@ -2856,7 +3349,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="16"/>
+      <c r="A15" s="18"/>
       <c r="B15" s="11" t="s">
         <v>88</v>
       </c>
@@ -2877,7 +3370,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="16"/>
+      <c r="A16" s="18"/>
       <c r="B16" s="11" t="s">
         <v>89</v>
       </c>
@@ -2898,7 +3391,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="16"/>
+      <c r="A17" s="18"/>
       <c r="B17" s="11" t="s">
         <v>90</v>
       </c>
@@ -2919,7 +3412,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="16"/>
+      <c r="A18" s="18"/>
       <c r="B18" s="11" t="s">
         <v>91</v>
       </c>
@@ -2940,7 +3433,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="16"/>
+      <c r="A19" s="18"/>
       <c r="B19" s="11" t="s">
         <v>92</v>
       </c>
@@ -2961,7 +3454,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="16"/>
+      <c r="A20" s="18"/>
       <c r="B20" s="11" t="s">
         <v>93</v>
       </c>
@@ -2982,7 +3475,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="16"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="11" t="s">
         <v>94</v>
       </c>
@@ -3003,7 +3496,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="16"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="11" t="s">
         <v>95</v>
       </c>
@@ -3024,7 +3517,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="16"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="11" t="s">
         <v>96</v>
       </c>
@@ -3045,7 +3538,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="16"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="11" t="s">
         <v>97</v>
       </c>
@@ -3066,7 +3559,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="16"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="11" t="s">
         <v>98</v>
       </c>
@@ -3087,7 +3580,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="16"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="11" t="s">
         <v>99</v>
       </c>
@@ -3108,7 +3601,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="16"/>
+      <c r="A27" s="18"/>
       <c r="B27" s="11" t="s">
         <v>100</v>
       </c>
@@ -3129,7 +3622,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="16"/>
+      <c r="A28" s="18"/>
       <c r="B28" s="11" t="s">
         <v>101</v>
       </c>
@@ -3150,7 +3643,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="16"/>
+      <c r="A29" s="18"/>
       <c r="B29" s="11" t="s">
         <v>170</v>
       </c>
@@ -3171,7 +3664,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="16"/>
+      <c r="A30" s="18"/>
       <c r="B30" s="11" t="s">
         <v>102</v>
       </c>
@@ -3192,7 +3685,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="16"/>
+      <c r="A31" s="18"/>
       <c r="B31" s="11" t="s">
         <v>103</v>
       </c>
@@ -3213,7 +3706,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" s="16"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="11" t="s">
         <v>104</v>
       </c>
@@ -3234,7 +3727,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="16"/>
+      <c r="A33" s="18"/>
       <c r="B33" s="11" t="s">
         <v>105</v>
       </c>
@@ -3255,7 +3748,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="16"/>
+      <c r="A34" s="18"/>
       <c r="B34" s="11" t="s">
         <v>106</v>
       </c>
@@ -3276,7 +3769,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="16"/>
+      <c r="A35" s="18"/>
       <c r="B35" s="11" t="s">
         <v>107</v>
       </c>
@@ -3297,7 +3790,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="16"/>
+      <c r="A36" s="18"/>
       <c r="B36" s="11" t="s">
         <v>108</v>
       </c>
@@ -3318,7 +3811,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="16"/>
+      <c r="A37" s="18"/>
       <c r="B37" s="11" t="s">
         <v>109</v>
       </c>
@@ -3339,7 +3832,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="16"/>
+      <c r="A38" s="18"/>
       <c r="B38" s="11" t="s">
         <v>110</v>
       </c>
@@ -3360,7 +3853,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="16"/>
+      <c r="A39" s="18"/>
       <c r="B39" s="11" t="s">
         <v>111</v>
       </c>
@@ -3381,7 +3874,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="16"/>
+      <c r="A40" s="18"/>
       <c r="B40" s="11" t="s">
         <v>112</v>
       </c>
@@ -3402,7 +3895,7 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="16"/>
+      <c r="A41" s="18"/>
       <c r="B41" s="11" t="s">
         <v>113</v>
       </c>
@@ -3423,7 +3916,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="16"/>
+      <c r="A42" s="18"/>
       <c r="B42" s="11" t="s">
         <v>114</v>
       </c>
@@ -3444,7 +3937,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="16"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="11" t="s">
         <v>115</v>
       </c>
@@ -3465,7 +3958,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="16"/>
+      <c r="A44" s="18"/>
       <c r="B44" s="11" t="s">
         <v>116</v>
       </c>
@@ -3486,7 +3979,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="16"/>
+      <c r="A45" s="18"/>
       <c r="B45" s="11" t="s">
         <v>117</v>
       </c>
@@ -3507,7 +4000,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="16"/>
+      <c r="A46" s="18"/>
       <c r="B46" s="11" t="s">
         <v>118</v>
       </c>
@@ -3528,7 +4021,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" s="16"/>
+      <c r="A47" s="18"/>
       <c r="B47" s="11" t="s">
         <v>119</v>
       </c>
@@ -3549,7 +4042,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="16"/>
+      <c r="A48" s="18"/>
       <c r="B48" s="11" t="s">
         <v>120</v>
       </c>
@@ -3570,7 +4063,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="16"/>
+      <c r="A49" s="18"/>
       <c r="B49" s="11" t="s">
         <v>121</v>
       </c>
@@ -3591,7 +4084,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50" s="16"/>
+      <c r="A50" s="18"/>
       <c r="B50" s="11" t="s">
         <v>122</v>
       </c>
@@ -3612,7 +4105,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A51" s="16"/>
+      <c r="A51" s="18"/>
       <c r="B51" s="11" t="s">
         <v>123</v>
       </c>
@@ -3633,7 +4126,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A52" s="16"/>
+      <c r="A52" s="18"/>
       <c r="B52" s="11" t="s">
         <v>172</v>
       </c>
@@ -3654,7 +4147,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A53" s="16"/>
+      <c r="A53" s="18"/>
       <c r="B53" s="11" t="s">
         <v>124</v>
       </c>
@@ -3675,7 +4168,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A54" s="16"/>
+      <c r="A54" s="18"/>
       <c r="B54" s="11" t="s">
         <v>125</v>
       </c>
@@ -3696,7 +4189,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55" s="16"/>
+      <c r="A55" s="18"/>
       <c r="B55" s="11" t="s">
         <v>126</v>
       </c>
@@ -3717,7 +4210,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" s="16"/>
+      <c r="A56" s="18"/>
       <c r="B56" s="11" t="s">
         <v>171</v>
       </c>
@@ -3746,7 +4239,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{708EFA42-0B00-4065-B708-67F0DF91E50F}">
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -3768,7 +4261,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>167</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -3779,7 +4272,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
+      <c r="A3" s="20"/>
       <c r="B3" s="7" t="s">
         <v>131</v>
       </c>
@@ -3788,7 +4281,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
+      <c r="A4" s="20"/>
       <c r="B4" s="7" t="s">
         <v>133</v>
       </c>
@@ -3797,7 +4290,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
+      <c r="A5" s="20"/>
       <c r="B5" s="7" t="s">
         <v>135</v>
       </c>
@@ -3806,7 +4299,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
+      <c r="A6" s="20"/>
       <c r="B6" s="7" t="s">
         <v>137</v>
       </c>
@@ -3815,7 +4308,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
+      <c r="A7" s="20"/>
       <c r="B7" s="7" t="s">
         <v>139</v>
       </c>
@@ -3824,7 +4317,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="18"/>
+      <c r="A8" s="20"/>
       <c r="B8" s="7" t="s">
         <v>141</v>
       </c>
@@ -3833,7 +4326,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
+      <c r="A9" s="20"/>
       <c r="B9" s="7" t="s">
         <v>143</v>
       </c>
@@ -3842,7 +4335,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="18"/>
+      <c r="A10" s="20"/>
       <c r="B10" s="7" t="s">
         <v>145</v>
       </c>
@@ -3851,7 +4344,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="7" t="s">
         <v>147</v>
       </c>
@@ -3860,7 +4353,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="18"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="7" t="s">
         <v>149</v>
       </c>
@@ -3869,7 +4362,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18"/>
+      <c r="A13" s="20"/>
       <c r="B13" s="7" t="s">
         <v>151</v>
       </c>
@@ -3878,7 +4371,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="18"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="7" t="s">
         <v>153</v>
       </c>
@@ -3887,7 +4380,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
+      <c r="A15" s="20"/>
       <c r="B15" s="7" t="s">
         <v>155</v>
       </c>
@@ -3896,7 +4389,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
+      <c r="A16" s="20"/>
       <c r="B16" s="7" t="s">
         <v>157</v>
       </c>
@@ -3905,7 +4398,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="18"/>
+      <c r="A17" s="20"/>
       <c r="B17" s="7" t="s">
         <v>159</v>
       </c>
@@ -3914,7 +4407,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="18"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="7" t="s">
         <v>161</v>
       </c>
@@ -3923,7 +4416,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="18"/>
+      <c r="A19" s="20"/>
       <c r="B19" s="7" t="s">
         <v>163</v>
       </c>
@@ -3932,7 +4425,7 @@
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="18"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="7" t="s">
         <v>165</v>
       </c>
@@ -3949,7 +4442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4EA2ECF-93A1-44B5-8689-5C67F3903905}">
   <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -3971,7 +4464,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>178</v>
       </c>
       <c r="B2" s="10" t="s">
@@ -3982,7 +4475,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="11" t="s">
         <v>175</v>
       </c>
@@ -3991,7 +4484,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="11" t="s">
         <v>177</v>
       </c>
@@ -4059,7 +4552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE41AAA-8C15-486A-A70D-82A4F7C63D41}">
   <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -4087,7 +4580,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>223</v>
       </c>
       <c r="B2" s="11">
@@ -4104,7 +4597,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="11">
         <v>2</v>
       </c>
@@ -4119,7 +4612,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="11">
         <v>3</v>
       </c>
@@ -4134,7 +4627,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="11">
         <v>4</v>
       </c>
@@ -4149,7 +4642,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="16"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="11">
         <v>5</v>
       </c>
@@ -4164,7 +4657,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="11">
         <v>6</v>
       </c>
@@ -4179,7 +4672,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="11">
         <v>7</v>
       </c>
@@ -4194,7 +4687,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="11">
         <v>8</v>
       </c>
@@ -4209,7 +4702,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="16"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="11">
         <v>9</v>
       </c>
@@ -4232,7 +4725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C23F822-AF2A-438F-A3B4-81476D3D8CF2}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -4257,7 +4750,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>209</v>
       </c>
       <c r="B2" s="11">
@@ -4271,7 +4764,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="11">
         <v>2</v>
       </c>
@@ -4283,7 +4776,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="11">
         <v>3</v>
       </c>
@@ -4295,7 +4788,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="11">
         <v>4</v>
       </c>
@@ -4307,7 +4800,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="16"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="11">
         <v>5</v>
       </c>
@@ -4319,7 +4812,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="11">
         <v>6</v>
       </c>
@@ -4331,7 +4824,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="11">
         <v>7</v>
       </c>
@@ -4376,7 +4869,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>227</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -4390,7 +4883,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="11" t="s">
         <v>18</v>
       </c>
@@ -4402,7 +4895,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="11" t="s">
         <v>19</v>
       </c>
@@ -4414,7 +4907,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="11" t="s">
         <v>20</v>
       </c>
@@ -4426,7 +4919,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="16"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="11" t="s">
         <v>22</v>
       </c>
@@ -4438,7 +4931,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="11" t="s">
         <v>23</v>
       </c>
@@ -4450,7 +4943,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="11" t="s">
         <v>25</v>
       </c>
@@ -4462,7 +4955,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="11" t="s">
         <v>27</v>
       </c>
@@ -4474,7 +4967,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="16"/>
+      <c r="A10" s="18"/>
       <c r="B10" s="11" t="s">
         <v>29</v>
       </c>
@@ -4486,7 +4979,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="16"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="11" t="s">
         <v>236</v>
       </c>
@@ -4507,6 +5000,209 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3A62034-87C0-4A5A-87E3-D16B6C010D9A}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="35.25" customWidth="1"/>
+    <col min="3" max="3" width="57.375" customWidth="1"/>
+    <col min="4" max="4" width="17.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="18"/>
+      <c r="B3" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="18"/>
+      <c r="B4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="18"/>
+      <c r="B5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="18"/>
+      <c r="B6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="18"/>
+      <c r="B7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="18"/>
+      <c r="B8" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="18"/>
+      <c r="B9" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="18"/>
+      <c r="B10" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="18"/>
+      <c r="B11" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="18"/>
+      <c r="B12" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="18"/>
+      <c r="B13" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="18"/>
+      <c r="B14" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="18"/>
+      <c r="B15" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A15"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34A8DB4A-58BD-4BB4-A87C-0E0F736365FB}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -4531,7 +5227,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>63</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -4545,7 +5241,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
+      <c r="A3" s="20"/>
       <c r="B3" s="7" t="s">
         <v>18</v>
       </c>
@@ -4557,7 +5253,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
+      <c r="A4" s="20"/>
       <c r="B4" s="7" t="s">
         <v>19</v>
       </c>
@@ -4569,7 +5265,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
+      <c r="A5" s="20"/>
       <c r="B5" s="7" t="s">
         <v>20</v>
       </c>
@@ -4581,7 +5277,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
+      <c r="A6" s="20"/>
       <c r="B6" s="7" t="s">
         <v>22</v>
       </c>
@@ -4593,7 +5289,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
+      <c r="A7" s="20"/>
       <c r="B7" s="7" t="s">
         <v>23</v>
       </c>
@@ -4605,7 +5301,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="18"/>
+      <c r="A8" s="20"/>
       <c r="B8" s="7" t="s">
         <v>25</v>
       </c>
@@ -4617,7 +5313,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
+      <c r="A9" s="20"/>
       <c r="B9" s="7" t="s">
         <v>27</v>
       </c>
@@ -4629,7 +5325,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="18"/>
+      <c r="A10" s="20"/>
       <c r="B10" s="7" t="s">
         <v>29</v>
       </c>
@@ -4649,7 +5345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FADAE7B0-3C6A-4E94-8340-AF191458A5A3}">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -4691,7 +5387,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="2">
@@ -4723,7 +5419,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="2">
         <v>2</v>
       </c>
@@ -4753,7 +5449,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="2">
         <v>4</v>
       </c>
@@ -4783,7 +5479,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="2">
         <v>4</v>
       </c>
@@ -4821,7 +5517,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCC641E5-B08E-4BF9-AF39-3E9AD6AB7462}">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -4863,7 +5559,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="2">
@@ -4895,7 +5591,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="2">
         <v>2</v>
       </c>
@@ -4925,7 +5621,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="2">
         <v>4</v>
       </c>
@@ -4955,7 +5651,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="2">
         <v>4</v>
       </c>
@@ -4993,7 +5689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51292F90-E6BB-47B7-8424-ED8217B2715E}">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -5035,7 +5731,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="2">
@@ -5067,7 +5763,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="2">
         <v>2</v>
       </c>
@@ -5097,7 +5793,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
+      <c r="A4" s="18"/>
       <c r="B4" s="2">
         <v>4</v>
       </c>
@@ -5127,7 +5823,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="2">
         <v>4</v>
       </c>
@@ -5165,7 +5861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B04511EA-F7FD-4F13-BC7F-6696711F80D1}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -5207,7 +5903,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="16" t="s">
         <v>45</v>
       </c>
       <c r="B2" s="2">
@@ -5239,7 +5935,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="20"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="2">
         <v>2</v>
       </c>
@@ -5269,7 +5965,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="20"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="2">
         <v>2</v>
       </c>
@@ -5299,7 +5995,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="20"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="2">
         <v>2</v>
       </c>
@@ -5329,7 +6025,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="2">
         <v>4</v>
       </c>
@@ -5359,7 +6055,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="2">
         <v>4</v>
       </c>
@@ -5389,7 +6085,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
+      <c r="A8" s="17"/>
       <c r="B8" s="2">
         <v>4</v>
       </c>
@@ -5419,7 +6115,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
+      <c r="A9" s="17"/>
       <c r="B9" s="2">
         <v>4</v>
       </c>
@@ -5457,7 +6153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D7A64D-D9EF-4E06-B43E-72FDFFD22334}">
   <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -5499,7 +6195,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B2" s="2">
@@ -5531,7 +6227,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="20"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="2">
         <v>4</v>
       </c>
@@ -5561,7 +6257,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="20"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="2">
         <v>4</v>
       </c>
@@ -5591,7 +6287,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="20"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="2">
         <v>4</v>
       </c>
@@ -5621,7 +6317,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="2">
         <v>8</v>
       </c>
@@ -5651,7 +6347,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="2">
         <v>8</v>
       </c>
@@ -5681,7 +6377,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
+      <c r="A8" s="17"/>
       <c r="B8" s="2">
         <v>8</v>
       </c>
@@ -5711,7 +6407,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
+      <c r="A9" s="17"/>
       <c r="B9" s="2">
         <v>8</v>
       </c>
@@ -5741,7 +6437,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="20"/>
+      <c r="A10" s="17"/>
       <c r="B10" s="2">
         <v>16</v>
       </c>
@@ -5771,7 +6467,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
+      <c r="A11" s="17"/>
       <c r="B11" s="2">
         <v>16</v>
       </c>
@@ -5801,7 +6497,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="20"/>
+      <c r="A12" s="17"/>
       <c r="B12" s="2">
         <v>16</v>
       </c>
@@ -5831,419 +6527,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="20"/>
-      <c r="B13" s="2">
-        <v>16</v>
-      </c>
-      <c r="C13" s="2">
-        <v>8</v>
-      </c>
-      <c r="D13" s="2">
-        <v>64</v>
-      </c>
-      <c r="E13" s="2">
-        <v>1024</v>
-      </c>
-      <c r="F13" s="2">
-        <v>16384</v>
-      </c>
-      <c r="G13" s="2">
-        <v>1</v>
-      </c>
-      <c r="H13" s="2">
-        <v>8</v>
-      </c>
-      <c r="I13" s="2">
-        <v>80</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:A13"/>
-  </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A658CE8-E02B-4E77-964D-75024B4BFBF4}">
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="53.375" customWidth="1"/>
-    <col min="5" max="5" width="11.625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B2" s="2">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>16</v>
-      </c>
-      <c r="E2" s="2">
-        <v>32</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1024</v>
-      </c>
-      <c r="G2" s="2">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2">
-        <v>8</v>
-      </c>
-      <c r="I2" s="2">
-        <v>320</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="20"/>
-      <c r="B3" s="2">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2">
-        <v>16</v>
-      </c>
-      <c r="E3" s="2">
-        <v>64</v>
-      </c>
-      <c r="F3" s="2">
-        <v>2048</v>
-      </c>
-      <c r="G3" s="2">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2">
-        <v>8</v>
-      </c>
-      <c r="I3" s="2">
-        <v>320</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="20"/>
-      <c r="B4" s="2">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2">
-        <v>4</v>
-      </c>
-      <c r="D4" s="2">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2">
-        <v>128</v>
-      </c>
-      <c r="F4" s="2">
-        <v>4096</v>
-      </c>
-      <c r="G4" s="2">
-        <v>1</v>
-      </c>
-      <c r="H4" s="2">
-        <v>8</v>
-      </c>
-      <c r="I4" s="2">
-        <v>320</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="20"/>
-      <c r="B5" s="2">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2">
-        <v>8</v>
-      </c>
-      <c r="D5" s="2">
-        <v>16</v>
-      </c>
-      <c r="E5" s="2">
-        <v>256</v>
-      </c>
-      <c r="F5" s="2">
-        <v>4096</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1</v>
-      </c>
-      <c r="H5" s="2">
-        <v>8</v>
-      </c>
-      <c r="I5" s="2">
-        <v>320</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
-      <c r="B6" s="2">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2">
-        <v>32</v>
-      </c>
-      <c r="E6" s="2">
-        <v>64</v>
-      </c>
-      <c r="F6" s="2">
-        <v>2048</v>
-      </c>
-      <c r="G6" s="2">
-        <v>1</v>
-      </c>
-      <c r="H6" s="2">
-        <v>8</v>
-      </c>
-      <c r="I6" s="2">
-        <v>160</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
-      <c r="B7" s="2">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2</v>
-      </c>
-      <c r="D7" s="2">
-        <v>32</v>
-      </c>
-      <c r="E7" s="2">
-        <v>128</v>
-      </c>
-      <c r="F7" s="2">
-        <v>4096</v>
-      </c>
-      <c r="G7" s="2">
-        <v>1</v>
-      </c>
-      <c r="H7" s="2">
-        <v>8</v>
-      </c>
-      <c r="I7" s="2">
-        <v>160</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
-      <c r="B8" s="2">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2">
-        <v>4</v>
-      </c>
-      <c r="D8" s="2">
-        <v>32</v>
-      </c>
-      <c r="E8" s="2">
-        <v>256</v>
-      </c>
-      <c r="F8" s="2">
-        <v>8192</v>
-      </c>
-      <c r="G8" s="2">
-        <v>1</v>
-      </c>
-      <c r="H8" s="2">
-        <v>8</v>
-      </c>
-      <c r="I8" s="2">
-        <v>160</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
-      <c r="B9" s="2">
-        <v>8</v>
-      </c>
-      <c r="C9" s="2">
-        <v>8</v>
-      </c>
-      <c r="D9" s="2">
-        <v>32</v>
-      </c>
-      <c r="E9" s="2">
-        <v>512</v>
-      </c>
-      <c r="F9" s="2">
-        <v>8192</v>
-      </c>
-      <c r="G9" s="2">
-        <v>1</v>
-      </c>
-      <c r="H9" s="2">
-        <v>8</v>
-      </c>
-      <c r="I9" s="2">
-        <v>160</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="20"/>
-      <c r="B10" s="2">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2">
-        <v>1</v>
-      </c>
-      <c r="D10" s="2">
-        <v>64</v>
-      </c>
-      <c r="E10" s="2">
-        <v>128</v>
-      </c>
-      <c r="F10" s="2">
-        <v>4096</v>
-      </c>
-      <c r="G10" s="2">
-        <v>1</v>
-      </c>
-      <c r="H10" s="2">
-        <v>8</v>
-      </c>
-      <c r="I10" s="2">
-        <v>80</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
-      <c r="B11" s="2">
-        <v>16</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2</v>
-      </c>
-      <c r="D11" s="2">
-        <v>64</v>
-      </c>
-      <c r="E11" s="2">
-        <v>256</v>
-      </c>
-      <c r="F11" s="2">
-        <v>8192</v>
-      </c>
-      <c r="G11" s="2">
-        <v>1</v>
-      </c>
-      <c r="H11" s="2">
-        <v>8</v>
-      </c>
-      <c r="I11" s="2">
-        <v>80</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="20"/>
-      <c r="B12" s="2">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2">
-        <v>4</v>
-      </c>
-      <c r="D12" s="2">
-        <v>64</v>
-      </c>
-      <c r="E12" s="2">
-        <v>512</v>
-      </c>
-      <c r="F12" s="2">
-        <v>16384</v>
-      </c>
-      <c r="G12" s="2">
-        <v>1</v>
-      </c>
-      <c r="H12" s="2">
-        <v>8</v>
-      </c>
-      <c r="I12" s="2">
-        <v>80</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="20"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="2">
         <v>16</v>
       </c>

</xml_diff>